<commit_message>
Clean the rows in the vacation requests file
</commit_message>
<xml_diff>
--- a/Ondrelle-Vacation-Requests.xlsx
+++ b/Ondrelle-Vacation-Requests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cyclotron-my.sharepoint.com/personal/mohamed_derhalli_cyclotron_com/Documents/Clients/Revlon/Ondrelle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_8173B3984EECA1B0D28A37769FC78751B67187A9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF01684F-026C-48F3-8557-8B805EC9C304}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_8173B3984EECA1B0D28A37769FC78751B67187A9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC9E3986-265B-4B46-8812-39CB4097E340}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -172,8 +172,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="VacationRequests" displayName="VacationRequests" ref="A1:D4">
-  <autoFilter ref="A1:D4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="VacationRequests" displayName="VacationRequests" ref="A1:D2" insertRow="1">
+  <autoFilter ref="A1:D2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Title"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="From Date"/>
@@ -469,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -496,18 +496,6 @@
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>